<commit_message>
Adjusting message Backend to Frontend
</commit_message>
<xml_diff>
--- a/backend/capital_consig_resultado.xlsx
+++ b/backend/capital_consig_resultado.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK19"/>
+  <dimension ref="A1:AF15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,7 +429,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Produto_y</t>
+          <t>Produto</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -569,35 +569,10 @@
       </c>
       <c r="AE1" t="inlineStr">
         <is>
-          <t>DIFERIMENTO</t>
+          <t>BONUS VIP</t>
         </is>
       </c>
       <c r="AF1" t="inlineStr">
-        <is>
-          <t>REPASSE DIFERIMENTO</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>SAFRA C. MENSAL</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>REPASSE SAFRA C. MENSAL</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>BONUS VIP</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
         <is>
           <t>REPASSE BONUS VIP</t>
         </is>
@@ -605,41 +580,41 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1055062</v>
+        <v>1044086</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SAFRA</t>
+          <t>CAPITAL CONSIG</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SIAPE-NOVO-1,75%-60-96</t>
+          <t>GOV PE_CC_EU QUERO_PL 70_CCC</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>FEDERAIS</t>
+          <t>GOVERNOS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>FEDERAL</t>
+          <t>ESTADUAL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FEDERAL SIAPE</t>
+          <t>GOV-PE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t>CARTÃO</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>96-96</t>
+          <t>48-48</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -674,7 +649,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -709,7 +684,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>3.000,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -719,7 +694,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -728,7 +703,7 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>314125</v>
+        <v>21513</v>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -742,40 +717,35 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="AD2" t="n">
-        <v>314125</v>
-      </c>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>3,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
+        <v>21513</v>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>2,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
         <is>
           <t>0,00 | 0,00 | 0,00</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1055044</v>
+        <v>1050433</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SAFRA</t>
+          <t>CAPITAL CONSIG</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PREF SAO PAULO-REFIN-1,75%-60-120</t>
+          <t>PREF SAO LUIS_EMP_F2_EU QUERO_PRD_CCC</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -790,17 +760,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>PREF. SAO PAULO SP</t>
+          <t>PREF. SAO LUIS MA</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>REFIN</t>
+          <t>NOVO</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>84-119</t>
+          <t>96-96</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -825,7 +795,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>3,000000</t>
+          <t>13,000000</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -840,17 +810,17 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2,100000</t>
+          <t>9,100000</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2,550000</t>
+          <t>12,350000</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2,850000</t>
+          <t>13,000000</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -870,7 +840,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>1.000,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -880,7 +850,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>24/03/2026</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -888,9 +858,7 @@
           <t>07/04/2026</t>
         </is>
       </c>
-      <c r="Z3" t="n">
-        <v>315091</v>
-      </c>
+      <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -906,44 +874,45 @@
           <t>LÍQUIDO</t>
         </is>
       </c>
-      <c r="AD3" t="n">
-        <v>315091</v>
-      </c>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>3,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>0,00 | 0,00 | 0,00</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1054962</v>
+        <v>1050434</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SAFRA</t>
+          <t>CAPITAL CONSIG</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MARINHA-NOVO-1,85%-60-72</t>
+          <t>PREF SAO LUIS_EMP_F3_EU QUERO_PRD_CCC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>FORCAS ARMADAS</t>
+          <t>PREFEITURAS</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>FORCAS ARMADAS</t>
+          <t>PREFEITURAS</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>MARINHA</t>
+          <t>PREF. SAO LUIS MA</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -953,7 +922,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>72-72</t>
+          <t>96-96</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -978,7 +947,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>5,000000</t>
+          <t>9,000000</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -988,22 +957,22 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>3,500000</t>
+          <t>6,300000</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>4,750000</t>
+          <t>8,550000</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>5,000000</t>
+          <t>9,000000</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -1023,7 +992,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>5.200,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -1033,7 +1002,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>24/03/2026</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -1041,9 +1010,7 @@
           <t>07/04/2026</t>
         </is>
       </c>
-      <c r="Z4" t="n">
-        <v>319060</v>
-      </c>
+      <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -1056,57 +1023,58 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>BRUTO</t>
-        </is>
-      </c>
-      <c r="AD4" t="n">
-        <v>319060</v>
-      </c>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
+          <t>LÍQUIDO</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>3,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>0,00 | 0,00 | 0,00</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1054927</v>
+        <v>1042978</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SAFRA</t>
+          <t>CAPITAL CONSIG</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>IPREM - APOSENTADO CONDICAO-PORT-1</t>
+          <t>SIAPE_CB_EUQUERO_CCC</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PREFEITURAS</t>
+          <t>FEDERAIS</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PREFEITURAS</t>
+          <t>FEDERAL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PREF. SAO PAULO SP</t>
+          <t>FEDERAL SIAPE</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>PORTABILIDADE</t>
+          <t>CARTÃO</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1-120</t>
+          <t>96-96</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1131,7 +1099,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0,000000</t>
+          <t>32,000000</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1141,22 +1109,22 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>0,000000</t>
+          <t>22,400000</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>0,000000</t>
+          <t>30,400000</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>0,000000</t>
+          <t>32,000000</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -1176,7 +1144,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>800,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
@@ -1186,7 +1154,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -1195,7 +1163,7 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>3408</v>
+        <v>19227</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -1209,57 +1177,60 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="AD5" t="n">
-        <v>3408</v>
-      </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
+        <v>19227</v>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>4,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>0,00 | 0,00 | 0,00</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1054971</v>
+        <v>1042976</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SAFRA</t>
+          <t>CAPITAL CONSIG</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MARINHA CONDICAO-PORT-1</t>
+          <t>SIAPE_CB_EUQUERO_PRD_CCC</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FORCAS ARMADAS</t>
+          <t>FEDERAIS</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FORCAS ARMADAS</t>
+          <t>FEDERAL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>MARINHA</t>
+          <t>FEDERAL SIAPE</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>PORTABILIDADE</t>
+          <t>CARTÃO</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1-72</t>
+          <t>96-96</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1284,7 +1255,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>0,000000</t>
+          <t>32,000000</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1294,22 +1265,22 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0,000000</t>
+          <t>22,400000</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>0,000000</t>
+          <t>30,400000</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>0,000000</t>
+          <t>32,000000</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1329,7 +1300,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>800,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1339,7 +1310,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1348,7 +1319,7 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>3822</v>
+        <v>19219</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1362,47 +1333,50 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="AD6" t="n">
-        <v>3822</v>
-      </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
+        <v>19219</v>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>4,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>0,00 | 0,00 | 0,00</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1054895</v>
+        <v>1044102</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SAFRA</t>
+          <t>CAPITAL CONSIG</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>INSS-NOVO-1,75%-72-96</t>
+          <t>GOV PBPREV_EMP_EU QUERO_CCC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>INSS</t>
+          <t>GOVERNOS</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>INSS</t>
+          <t>ESTADUAL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>INSS</t>
+          <t>GOV-PB</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1437,7 +1411,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>3,000000</t>
+          <t>11,000000</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1447,22 +1421,22 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2,100000</t>
+          <t>7,700000</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2,850000</t>
+          <t>10,450000</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>3,000000</t>
+          <t>11,000000</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1482,7 +1456,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>1.000,00-100.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1492,7 +1466,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1501,7 +1475,7 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>314120</v>
+        <v>21485</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -1515,52 +1489,55 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="AD7" t="n">
-        <v>314120</v>
-      </c>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
+        <v>21485</v>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>3,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>0,00 | 0,00 | 0,00</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1054886</v>
+        <v>1042975</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SAFRA</t>
+          <t>CAPITAL CONSIG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GOV SP SPPREV-REFIN_PORT-1,75%-96</t>
+          <t>SIAPE_CB_EUQUERO_EXCEÇÃO_CCC</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GOVERNOS</t>
+          <t>FEDERAIS</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ESTADUAL</t>
+          <t>FEDERAL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>GOV-SP</t>
+          <t>FEDERAL SIAPE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>PORTAB/REFIN</t>
+          <t>CARTÃO</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1590,7 +1567,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>3,000000</t>
+          <t>32,000000</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1600,22 +1577,22 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2,100000</t>
+          <t>22,400000</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2,550000</t>
+          <t>30,400000</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2,850000</t>
+          <t>32,000000</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1635,7 +1612,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>5.000,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1645,7 +1622,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -1654,7 +1631,7 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>315082</v>
+        <v>19218</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -1668,57 +1645,60 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="AD8" t="n">
-        <v>315082</v>
-      </c>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
+        <v>19218</v>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>4,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>0,00 | 0,00 | 0,00</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1054984</v>
+        <v>1042977</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SAFRA</t>
+          <t>CAPITAL CONSIG</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MARINHA-REFIN_PORT-1,75%-72-72</t>
+          <t>SIAPE_CB_EUQUERO_PRD_EXCEÇÃO_CCC</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FORCAS ARMADAS</t>
+          <t>FEDERAIS</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>FORCAS ARMADAS</t>
+          <t>FEDERAL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>MARINHA</t>
+          <t>FEDERAL SIAPE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>PORTAB/REFIN</t>
+          <t>CARTÃO</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>72-72</t>
+          <t>96-96</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1743,7 +1723,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2,000000</t>
+          <t>32,000000</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1753,22 +1733,22 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>1,400000</t>
+          <t>22,400000</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1,700000</t>
+          <t>30,400000</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1,900000</t>
+          <t>32,000000</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1788,7 +1768,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2.000,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1798,7 +1778,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -1807,7 +1787,7 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>319072</v>
+        <v>19220</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
@@ -1821,15 +1801,15 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="AD9" t="n">
-        <v>319072</v>
+        <v>19220</v>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>1,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+          <t>4,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -1837,11 +1817,6 @@
           <t>0,00 | 0,00 | 0,00</t>
         </is>
       </c>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
@@ -1850,30 +1825,34 @@
           <t>CAPITAL CONSIG</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GOV PE_CC_EU QUERO_PL 70_CCC</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PREFEITURAS</t>
+          <t>GOVERNOS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>PREFEITURAS</t>
+          <t>ESTADUAL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PREF. SAO PAULO SP</t>
+          <t>GOV-PE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t>CARTÃO</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>60-121</t>
+          <t>47-47</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1897,7 +1876,7 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -1910,13 +1889,13 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>4.199999999999999</v>
+        <v>3.5</v>
       </c>
       <c r="Q10" t="n">
-        <v>5.699999999999999</v>
+        <v>4.75</v>
       </c>
       <c r="R10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1935,7 +1914,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2.000,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1950,7 +1929,7 @@
       </c>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="n">
-        <v>293537</v>
+        <v>21513</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1968,27 +1947,14 @@
         </is>
       </c>
       <c r="AD10" t="n">
-        <v>293537</v>
+        <v>21513</v>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>0,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+          <t>2,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
-        <is>
-          <t>0,00 | 0,00 | 0,00</t>
-        </is>
-      </c>
-      <c r="AG10" t="inlineStr"/>
-      <c r="AH10" t="inlineStr"/>
-      <c r="AI10" t="inlineStr">
-        <is>
-          <t>IPREM - ATIVO-NOVO-1,85%-60-120</t>
-        </is>
-      </c>
-      <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr">
         <is>
           <t>0,00 | 0,00 | 0,00</t>
         </is>
@@ -2001,30 +1967,34 @@
           <t>CAPITAL CONSIG</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SIAPE_CB_EUQUERO_CCC</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PREFEITURAS</t>
+          <t>FEDERAIS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PREFEITURAS</t>
+          <t>FEDERAL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PREF. BELO HORIZONTE MG</t>
+          <t>FEDERAL SIAPE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t>CARTÃO</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>120-171</t>
+          <t>100-100</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -2048,7 +2018,7 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -2061,13 +2031,13 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>4.199999999999999</v>
+        <v>22.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>5.699999999999999</v>
+        <v>30.4</v>
       </c>
       <c r="R11" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -2086,7 +2056,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>5.200,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -2101,7 +2071,7 @@
       </c>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="n">
-        <v>296622</v>
+        <v>19227</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -2119,27 +2089,14 @@
         </is>
       </c>
       <c r="AD11" t="n">
-        <v>296622</v>
+        <v>19227</v>
       </c>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>2,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+          <t>4,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
-        <is>
-          <t>0,00 | 0,00 | 0,00</t>
-        </is>
-      </c>
-      <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="inlineStr"/>
-      <c r="AI11" t="inlineStr">
-        <is>
-          <t>PREF BELO HORIZONTE-NOVO-2,09%-120-120</t>
-        </is>
-      </c>
-      <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr">
         <is>
           <t>0,00 | 0,00 | 0,00</t>
         </is>
@@ -2152,7 +2109,11 @@
           <t>CAPITAL CONSIG</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SIAPE_CB_EUQUERO_PRD_CCC</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>FEDERAIS</t>
@@ -2170,12 +2131,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t>CARTÃO</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>98-98</t>
+          <t>99-99</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2199,7 +2160,7 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -2212,13 +2173,13 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>3.5</v>
+        <v>22.4</v>
       </c>
       <c r="Q12" t="n">
-        <v>4.75</v>
+        <v>30.4</v>
       </c>
       <c r="R12" t="n">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -2237,7 +2198,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>3.000,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
@@ -2252,7 +2213,7 @@
       </c>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="n">
-        <v>314125</v>
+        <v>19219</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -2270,27 +2231,14 @@
         </is>
       </c>
       <c r="AD12" t="n">
-        <v>314125</v>
+        <v>19219</v>
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>0,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+          <t>4,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
-        <is>
-          <t>0,00 | 0,00 | 0,00</t>
-        </is>
-      </c>
-      <c r="AG12" t="inlineStr"/>
-      <c r="AH12" t="inlineStr"/>
-      <c r="AI12" t="inlineStr">
-        <is>
-          <t>SIAPE-NOVO-1,75%-60-96</t>
-        </is>
-      </c>
-      <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr">
         <is>
           <t>0,00 | 0,00 | 0,00</t>
         </is>
@@ -2303,20 +2251,24 @@
           <t>CAPITAL CONSIG</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GOV PBPREV_EMP_EU QUERO_CCC</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>FORCAS ARMADAS</t>
+          <t>GOVERNOS</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FORCAS ARMADAS</t>
+          <t>ESTADUAL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>MARINHA</t>
+          <t>GOV-PB</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2326,7 +2278,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>60-171</t>
+          <t>96-96</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2350,7 +2302,7 @@
         </is>
       </c>
       <c r="M13" t="n">
-        <v>2.5</v>
+        <v>10</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -2363,13 +2315,13 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>1.75</v>
+        <v>7</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.375</v>
+        <v>9.5</v>
       </c>
       <c r="R13" t="n">
-        <v>2.5</v>
+        <v>10</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -2388,7 +2340,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>5.200,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -2403,7 +2355,7 @@
       </c>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="n">
-        <v>319061</v>
+        <v>21485</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -2421,27 +2373,14 @@
         </is>
       </c>
       <c r="AD13" t="n">
-        <v>319061</v>
+        <v>21485</v>
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>0,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+          <t>3,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
-        <is>
-          <t>0,00 | 0,00 | 0,00</t>
-        </is>
-      </c>
-      <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr">
-        <is>
-          <t>MARINHA-NOVO-1,79%-60-72</t>
-        </is>
-      </c>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr">
         <is>
           <t>0,00 | 0,00 | 0,00</t>
         </is>
@@ -2454,7 +2393,11 @@
           <t>CAPITAL CONSIG</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SIAPE_CB_EUQUERO_EXCEÇÃO_CCC</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>FEDERAIS</t>
@@ -2472,12 +2415,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>REFIN_PORT</t>
+          <t>CARTÃO</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>120-120</t>
+          <t>96-96</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -2501,7 +2444,7 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -2514,13 +2457,13 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>6.3</v>
+        <v>4.199999999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>8.549999999999999</v>
+        <v>5.699999999999999</v>
       </c>
       <c r="R14" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -2539,7 +2482,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>15.000,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -2554,7 +2497,7 @@
       </c>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="n">
-        <v>319175</v>
+        <v>19218</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
@@ -2572,27 +2515,14 @@
         </is>
       </c>
       <c r="AD14" t="n">
-        <v>319175</v>
+        <v>19218</v>
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>0,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+          <t>4,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
-        <is>
-          <t>0,00 | 0,00 | 0,00</t>
-        </is>
-      </c>
-      <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr"/>
-      <c r="AI14" t="inlineStr">
-        <is>
-          <t>SIAPE-REFIN_PORT-1,59%-96-96</t>
-        </is>
-      </c>
-      <c r="AJ14" t="inlineStr"/>
-      <c r="AK14" t="inlineStr">
         <is>
           <t>0,00 | 0,00 | 0,00</t>
         </is>
@@ -2602,37 +2532,37 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SAFRA</t>
+          <t>CAPITAL CONSIG</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>IPREM - APOSENTADO CONDICAO-PORT-1</t>
+          <t>SIAPE_CB_EUQUERO_PRD_EXCEÇÃO_CCC</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>PREFEITURAS</t>
+          <t>FEDERAIS</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>PREFEITURAS</t>
+          <t>FEDERAL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PREF. SAO PAULO SP</t>
+          <t>FEDERAL SIAPE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>PORTABILIDADE</t>
+          <t>CARTÃO</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1-120</t>
+          <t>96-96</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2656,7 +2586,7 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -2665,17 +2595,17 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>8.399999999999999</v>
+        <v>2.8</v>
       </c>
       <c r="Q15" t="n">
-        <v>11.4</v>
+        <v>3.8</v>
       </c>
       <c r="R15" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -2694,7 +2624,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>800,00-200.000,00-LÍQUIDO</t>
+          <t>0,00-100.000,00-LÍQUIDO</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -2709,7 +2639,7 @@
       </c>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="n">
-        <v>3408</v>
+        <v>19220</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -2723,583 +2653,22 @@
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>BRUTO</t>
+          <t>LÍQUIDO</t>
         </is>
       </c>
       <c r="AD15" t="n">
-        <v>3408</v>
-      </c>
-      <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr"/>
-      <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
-      <c r="AK15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>SAFRA</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>MARINHA CONDICAO-PORT-1</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>FORCAS ARMADAS</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>FORCAS ARMADAS</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>MARINHA</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>PORTABILIDADE</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>1-72</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>0-80</t>
-        </is>
-      </c>
-      <c r="M16" t="n">
-        <v>10</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>BRUTO</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="R16" t="n">
-        <v>10</v>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>0,000000000</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>0,000000</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>0,000000</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>800,00-200.000,00-LÍQUIDO</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>07/04/2026</t>
-        </is>
-      </c>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="n">
-        <v>3822</v>
-      </c>
-      <c r="AA16" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="AB16" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="AC16" t="inlineStr">
-        <is>
-          <t>BRUTO</t>
-        </is>
-      </c>
-      <c r="AD16" t="n">
-        <v>3822</v>
-      </c>
-      <c r="AE16" t="inlineStr"/>
-      <c r="AF16" t="inlineStr"/>
-      <c r="AG16" t="inlineStr"/>
-      <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>SAFRA</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>INSS-NOVO-1,75%-72-96</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>INSS</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>INSS</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>INSS</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>NOVO</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>96-96</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>0-80</t>
-        </is>
-      </c>
-      <c r="M17" t="n">
-        <v>4</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>BRUTO</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="R17" t="n">
-        <v>4</v>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>0,000000000</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>0,000000</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>0,000000</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>1.000,00-100.000,00-LÍQUIDO</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>07/04/2026</t>
-        </is>
-      </c>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="n">
-        <v>314120</v>
-      </c>
-      <c r="AA17" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="AB17" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="AC17" t="inlineStr">
-        <is>
-          <t>BRUTO</t>
-        </is>
-      </c>
-      <c r="AD17" t="n">
-        <v>314120</v>
-      </c>
-      <c r="AE17" t="inlineStr"/>
-      <c r="AF17" t="inlineStr"/>
-      <c r="AG17" t="inlineStr"/>
-      <c r="AH17" t="inlineStr"/>
-      <c r="AI17" t="inlineStr"/>
-      <c r="AJ17" t="inlineStr"/>
-      <c r="AK17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SAFRA</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>GOV SP SPPREV-REFIN_PORT-1,75%-96</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>GOVERNOS</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>ESTADUAL</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>GOV-SP</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>PORTAB/REFIN</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>96-96</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>0-80</t>
-        </is>
-      </c>
-      <c r="M18" t="n">
-        <v>9</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>BRUTO</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>8.549999999999999</v>
-      </c>
-      <c r="R18" t="n">
-        <v>9</v>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>0,000000000</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>0,000000</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>0,000000</t>
-        </is>
-      </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>5.000,00-200.000,00-LÍQUIDO</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>07/04/2026</t>
-        </is>
-      </c>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="n">
-        <v>315082</v>
-      </c>
-      <c r="AA18" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="AB18" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="AC18" t="inlineStr">
-        <is>
-          <t>BRUTO</t>
-        </is>
-      </c>
-      <c r="AD18" t="n">
-        <v>315082</v>
-      </c>
-      <c r="AE18" t="inlineStr"/>
-      <c r="AF18" t="inlineStr"/>
-      <c r="AG18" t="inlineStr"/>
-      <c r="AH18" t="inlineStr"/>
-      <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" t="inlineStr"/>
-      <c r="AK18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SAFRA</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>MARINHA-REFIN_PORT-1,75%-72-72</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>FORCAS ARMADAS</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>FORCAS ARMADAS</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>MARINHA</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>PORTAB/REFIN</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>72-72</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>0-80</t>
-        </is>
-      </c>
-      <c r="M19" t="n">
-        <v>6</v>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>BRUTO</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
-        <v>4.199999999999999</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>5.699999999999999</v>
-      </c>
-      <c r="R19" t="n">
-        <v>6</v>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>0,000000000</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>0,000000</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>0,000000</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>2.000,00-200.000,00-LÍQUIDO</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>0,00-0,00</t>
-        </is>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>07/04/2026</t>
-        </is>
-      </c>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="n">
-        <v>319072</v>
-      </c>
-      <c r="AA19" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="AB19" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="AC19" t="inlineStr">
-        <is>
-          <t>BRUTO</t>
-        </is>
-      </c>
-      <c r="AD19" t="n">
-        <v>319072</v>
-      </c>
-      <c r="AE19" t="inlineStr">
-        <is>
-          <t>1,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
-        </is>
-      </c>
-      <c r="AF19" t="inlineStr">
+        <v>19220</v>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>4,00 | LIQUIDO | 0,00 | NÃO | SEM VIG. INÍCIO | SEM VIG. TÉRMINO</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
         <is>
           <t>0,00 | 0,00 | 0,00</t>
         </is>
       </c>
-      <c r="AG19" t="inlineStr"/>
-      <c r="AH19" t="inlineStr"/>
-      <c r="AI19" t="inlineStr"/>
-      <c r="AJ19" t="inlineStr"/>
-      <c r="AK19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>